<commit_message>
Phase 1: Ergebnis des Tenant-Checks eingearbeitet
- Test-TenantReadiness: RMS-Vorlagen mit GUID ausgeben und lokalisierte
  Namen (Encrypt = Verschlüsseln) erkennen; SPO-Modul unter PowerShell 7
  mit vollem Pfad importieren.
- Testkonten und Doku an die geprüften Gruppen angepasst: Debra Berger ist
  nur im Finance Team, MOD Administrator in allen drei Gruppen.
- Anleitung: falsche Angabe zu 'Confidential \ All Employees' korrigiert.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B9kfFEfvigtmrSNC6uJaHV
</commit_message>
<xml_diff>
--- a/Demo Dokumente/Testprotokoll-Purview-Demos.xlsx
+++ b/Demo Dokumente/Testprotokoll-Purview-Demos.xlsx
@@ -576,12 +576,12 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Finance Team, Leadership</t>
+          <t>Finance Team</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Confidential-Finance; hat über Leadership auch Rechte auf Legal und Strictly-Confidential-Intern — kein Negativtest für Legal</t>
+          <t>Confidential-Finance; zugleich Negativtest für Legal und Strictly-Confidential-Intern</t>
         </is>
       </c>
     </row>

</xml_diff>